<commit_message>
Update vegetable recommendations Excel file and thumbnail image for improved content and visuals.
</commit_message>
<xml_diff>
--- a/files/vegetable-recommendations.xlsx
+++ b/files/vegetable-recommendations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jusep\Desktop\PROJECTS\amia-microsite.github.io\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565D54EF-4341-41EE-B51C-3235AC1CAE8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F444883F-A38C-4EC9-87CD-A4C66B347810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7635" yWindow="2325" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="4" xr2:uid="{E2D1DC89-D079-3B4D-864B-8CE149E3E279}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E2D1DC89-D079-3B4D-864B-8CE149E3E279}"/>
   </bookViews>
   <sheets>
     <sheet name="Vegetable_10Day(Municipal)" sheetId="9" r:id="rId1"/>
@@ -1193,7 +1193,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1360,38 +1360,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="7" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="7" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1404,6 +1377,36 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="7" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -1751,14 +1754,14 @@
       <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58" t="s">
+      <c r="E1" s="64"/>
+      <c r="F1" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="58"/>
+      <c r="G1" s="64"/>
       <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1783,7 +1786,7 @@
       <c r="A3" s="53" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="60" t="s">
         <v>77</v>
       </c>
       <c r="C3" s="30" t="s">
@@ -1813,7 +1816,7 @@
         <v>113</v>
       </c>
       <c r="E4" s="56"/>
-      <c r="F4" s="66" t="s">
+      <c r="F4" s="58" t="s">
         <v>115</v>
       </c>
       <c r="G4" s="30"/>
@@ -1833,7 +1836,7 @@
         <v>116</v>
       </c>
       <c r="E5" s="56"/>
-      <c r="F5" s="66" t="s">
+      <c r="F5" s="58" t="s">
         <v>108</v>
       </c>
       <c r="G5" s="30"/>
@@ -1843,7 +1846,7 @@
       <c r="A6" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="69" t="s">
+      <c r="B6" s="60" t="s">
         <v>71</v>
       </c>
       <c r="C6" s="30" t="s">
@@ -1891,7 +1894,7 @@
       <c r="A9" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="69" t="s">
+      <c r="B9" s="60" t="s">
         <v>78</v>
       </c>
       <c r="C9" s="30" t="s">
@@ -1939,7 +1942,7 @@
       <c r="A12" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="69" t="s">
+      <c r="B12" s="60" t="s">
         <v>72</v>
       </c>
       <c r="C12" s="30" t="s">
@@ -1987,7 +1990,7 @@
       <c r="A15" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="69" t="s">
+      <c r="B15" s="60" t="s">
         <v>73</v>
       </c>
       <c r="C15" s="30" t="s">
@@ -2035,7 +2038,7 @@
       <c r="A18" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="B18" s="69" t="s">
+      <c r="B18" s="60" t="s">
         <v>74</v>
       </c>
       <c r="C18" s="30" t="s">
@@ -2083,7 +2086,7 @@
       <c r="A21" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="69" t="s">
+      <c r="B21" s="60" t="s">
         <v>13</v>
       </c>
       <c r="C21" s="30" t="s">
@@ -2131,7 +2134,7 @@
       <c r="A24" s="50" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="69" t="s">
+      <c r="B24" s="60" t="s">
         <v>79</v>
       </c>
       <c r="C24" s="30" t="s">
@@ -2179,7 +2182,7 @@
       <c r="A27" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="70" t="s">
+      <c r="B27" s="61" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="29" t="s">
@@ -2227,7 +2230,7 @@
       <c r="A30" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="B30" s="70" t="s">
+      <c r="B30" s="61" t="s">
         <v>67</v>
       </c>
       <c r="C30" s="29" t="s">
@@ -2323,7 +2326,7 @@
       <c r="A36" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="B36" s="70" t="s">
+      <c r="B36" s="61" t="s">
         <v>76</v>
       </c>
       <c r="C36" s="29" t="s">
@@ -2371,7 +2374,7 @@
       <c r="A39" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="B39" s="71" t="s">
+      <c r="B39" s="62" t="s">
         <v>11</v>
       </c>
       <c r="C39" s="26" t="s">
@@ -2515,7 +2518,7 @@
       <c r="A48" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="B48" s="71" t="s">
+      <c r="B48" s="62" t="s">
         <v>82</v>
       </c>
       <c r="C48" s="26" t="s">
@@ -2563,7 +2566,7 @@
       <c r="A51" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="72" t="s">
+      <c r="B51" s="63" t="s">
         <v>81</v>
       </c>
       <c r="C51" s="28" t="s">
@@ -2608,7 +2611,7 @@
       <c r="A54" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="B54" s="72" t="s">
+      <c r="B54" s="63" t="s">
         <v>13</v>
       </c>
       <c r="C54" s="28" t="s">
@@ -3394,14 +3397,14 @@
       <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58" t="s">
+      <c r="E1" s="64"/>
+      <c r="F1" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="58"/>
+      <c r="G1" s="64"/>
       <c r="H1" s="11"/>
       <c r="I1" s="14"/>
     </row>
@@ -5506,16 +5509,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="67" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
       <c r="J1" s="52"/>
       <c r="K1" s="52"/>
       <c r="L1" s="52"/>
@@ -5526,16 +5529,16 @@
       <c r="Q1" s="52"/>
     </row>
     <row r="2" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
       <c r="J2" s="55"/>
       <c r="K2" s="55"/>
       <c r="L2" s="55"/>
@@ -5546,162 +5549,162 @@
       <c r="Q2" s="55"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="65" t="s">
         <v>117</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
     </row>
     <row r="4" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="70" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
-      <c r="H4" s="59"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="65" t="s">
         <v>122</v>
       </c>
-      <c r="C5" s="59"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
-      <c r="H5" s="59"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="68" t="s">
         <v>130</v>
       </c>
-      <c r="C6" s="61"/>
-      <c r="D6" s="61"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
-      <c r="G6" s="61"/>
-      <c r="H6" s="61"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="68"/>
+      <c r="F6" s="68"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="68"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="60" t="s">
+      <c r="A9" s="69" t="s">
         <v>119</v>
       </c>
-      <c r="B9" s="60"/>
-      <c r="C9" s="60"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="60"/>
-      <c r="F9" s="60"/>
-      <c r="G9" s="60"/>
-      <c r="H9" s="60"/>
+      <c r="B9" s="69"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="69"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="69"/>
+      <c r="H9" s="69"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="59" t="s">
+      <c r="B10" s="65" t="s">
         <v>120</v>
       </c>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="59"/>
+      <c r="C10" s="65"/>
+      <c r="D10" s="65"/>
+      <c r="E10" s="65"/>
+      <c r="F10" s="65"/>
+      <c r="G10" s="65"/>
+      <c r="H10" s="65"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="63" t="s">
+      <c r="B11" s="70" t="s">
         <v>121</v>
       </c>
-      <c r="C11" s="59"/>
-      <c r="D11" s="59"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="59"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="61" t="s">
+      <c r="B12" s="66" t="s">
         <v>129</v>
       </c>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
-      <c r="G12" s="61"/>
-      <c r="H12" s="61"/>
+      <c r="C12" s="66"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="66"/>
+      <c r="G12" s="66"/>
+      <c r="H12" s="66"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A15" s="60" t="s">
+      <c r="A15" s="69" t="s">
         <v>123</v>
       </c>
-      <c r="B15" s="60"/>
-      <c r="C15" s="60"/>
-      <c r="D15" s="60"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="60"/>
-      <c r="H15" s="60"/>
+      <c r="B15" s="69"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="69"/>
+      <c r="E15" s="69"/>
+      <c r="F15" s="69"/>
+      <c r="G15" s="69"/>
+      <c r="H15" s="69"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="59" t="s">
+      <c r="B16" s="65" t="s">
         <v>124</v>
       </c>
-      <c r="C16" s="59"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="59"/>
-      <c r="H16" s="59"/>
+      <c r="C16" s="65"/>
+      <c r="D16" s="65"/>
+      <c r="E16" s="65"/>
+      <c r="F16" s="65"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="65"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="66" t="s">
         <v>128</v>
       </c>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
+      <c r="C17" s="66"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="66"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="60" t="s">
+      <c r="A20" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="60"/>
+      <c r="B20" s="69"/>
+      <c r="C20" s="69"/>
+      <c r="D20" s="69"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="69"/>
+      <c r="G20" s="69"/>
+      <c r="H20" s="69"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="60" t="s">
+      <c r="A23" s="69" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="60"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="60"/>
+      <c r="B23" s="69"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="69"/>
+      <c r="E23" s="69"/>
+      <c r="F23" s="69"/>
+      <c r="G23" s="69"/>
+      <c r="H23" s="69"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="61" t="s">
+      <c r="B24" s="66" t="s">
         <v>127</v>
       </c>
-      <c r="C24" s="61"/>
-      <c r="D24" s="61"/>
-      <c r="E24" s="61"/>
-      <c r="F24" s="61"/>
-      <c r="G24" s="61"/>
-      <c r="H24" s="61"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
+      <c r="F24" s="66"/>
+      <c r="G24" s="66"/>
+      <c r="H24" s="66"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B39" s="57"/>
@@ -5713,26 +5716,26 @@
       <c r="H39" s="57"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="59" t="s">
+      <c r="B40" s="65" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="59"/>
-      <c r="D40" s="59"/>
-      <c r="E40" s="59"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="59"/>
-      <c r="H40" s="59"/>
+      <c r="C40" s="65"/>
+      <c r="D40" s="65"/>
+      <c r="E40" s="65"/>
+      <c r="F40" s="65"/>
+      <c r="G40" s="65"/>
+      <c r="H40" s="65"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="61" t="s">
+      <c r="B41" s="66" t="s">
         <v>109</v>
       </c>
-      <c r="C41" s="61"/>
-      <c r="D41" s="61"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="61"/>
-      <c r="G41" s="61"/>
-      <c r="H41" s="61"/>
+      <c r="C41" s="66"/>
+      <c r="D41" s="66"/>
+      <c r="E41" s="66"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="66"/>
+      <c r="H41" s="66"/>
     </row>
     <row r="42" spans="1:8" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A42" s="57" t="s">
@@ -5742,9 +5745,6 @@
     <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B24:H24"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B40:H40"/>
@@ -5760,6 +5760,9 @@
     <mergeCell ref="B11:H11"/>
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B24:H24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5775,10 +5778,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="59" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="67" t="s">
+      <c r="B1" s="59" t="s">
         <v>101</v>
       </c>
     </row>
@@ -5830,10 +5833,10 @@
     </row>
     <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:2" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="71" t="s">
         <v>88</v>
       </c>
-      <c r="B10" s="68"/>
+      <c r="B10" s="71"/>
     </row>
     <row r="11" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="51" t="s">
@@ -5869,10 +5872,10 @@
     </row>
     <row r="15" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="68" t="s">
+      <c r="A16" s="71" t="s">
         <v>91</v>
       </c>
-      <c r="B16" s="68"/>
+      <c r="B16" s="71"/>
     </row>
     <row r="17" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="51" t="s">
@@ -5957,14 +5960,14 @@
       <c r="A1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64" t="s">
+      <c r="C1" s="72"/>
+      <c r="D1" s="72" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="64"/>
+      <c r="E1" s="72"/>
       <c r="F1" s="11"/>
       <c r="G1" s="14"/>
     </row>
@@ -6998,14 +7001,14 @@
       <c r="A1" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65" t="s">
+      <c r="C1" s="73"/>
+      <c r="D1" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="65"/>
+      <c r="E1" s="73"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="20"/>

</xml_diff>